<commit_message>
Update card database to new xlsx schema (drop orange, add yellow, special-text support)
</commit_message>
<xml_diff>
--- a/dragon_card_sets.xlsx
+++ b/dragon_card_sets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c106bd21665f125/Desktop/Queue/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c106bd21665f125/Desktop/Domino/SomethingSomethingDragons/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="11_E069DF57A4384892C03CCB8E22CF3148C9D4FB8C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBF0EEFC-AC65-4D3F-A3F1-C6A81751A7B0}"/>
+  <xr:revisionPtr revIDLastSave="376" documentId="11_E069DF57A4384892C03CCB8E22CF3148C9D4FB8C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08409FCC-11EA-4974-962B-7163362D285A}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11175" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11175" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Green Dragon" sheetId="6" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="129">
   <si>
     <t>Card #</t>
   </si>
@@ -33,12 +33,6 @@
     <t>Card Name</t>
   </si>
   <si>
-    <t>Card Type</t>
-  </si>
-  <si>
-    <t>Base Effect</t>
-  </si>
-  <si>
     <t>Boost Effect</t>
   </si>
   <si>
@@ -69,33 +63,18 @@
     <t>Flame Bolt</t>
   </si>
   <si>
-    <t>Deal +3 damage</t>
-  </si>
-  <si>
     <t>Burning Charge</t>
   </si>
   <si>
     <t>Bloodfire Slash</t>
   </si>
   <si>
-    <t>Deal 5 damage</t>
-  </si>
-  <si>
     <t>Inferno Wings</t>
   </si>
   <si>
-    <t>Gain 4 movement</t>
-  </si>
-  <si>
     <t>Dragon Rage</t>
   </si>
   <si>
-    <t>Utility</t>
-  </si>
-  <si>
-    <t>Draw 1 card</t>
-  </si>
-  <si>
     <t>Scorching Arc</t>
   </si>
   <si>
@@ -105,15 +84,9 @@
     <t>Molten Scales</t>
   </si>
   <si>
-    <t>Defense</t>
-  </si>
-  <si>
     <t>Phoenix Dive</t>
   </si>
   <si>
-    <t>Heal 2</t>
-  </si>
-  <si>
     <t>Cinderstorm</t>
   </si>
   <si>
@@ -123,15 +96,9 @@
     <t>Execution Strike</t>
   </si>
   <si>
-    <t>Deal 4 damage</t>
-  </si>
-  <si>
     <t>Hellkite Rush</t>
   </si>
   <si>
-    <t>Gain 5 movement</t>
-  </si>
-  <si>
     <t>Ashen Frenzy</t>
   </si>
   <si>
@@ -141,48 +108,27 @@
     <t>Mystic Flow</t>
   </si>
   <si>
-    <t>Gain 2 magic</t>
-  </si>
-  <si>
     <t>Arcane Step</t>
   </si>
   <si>
-    <t>Gain 3 movement</t>
-  </si>
-  <si>
-    <t>Gain 1 magic</t>
-  </si>
-  <si>
     <t>Mana Surge</t>
   </si>
   <si>
-    <t>Draw 2 cards</t>
-  </si>
-  <si>
     <t>Frost Sigil</t>
   </si>
   <si>
-    <t>Deal 2 damage</t>
-  </si>
-  <si>
     <t>Meditation</t>
   </si>
   <si>
     <t>Blink</t>
   </si>
   <si>
-    <t>Ignore enemy zones this turn</t>
-  </si>
-  <si>
     <t>Spell Recall</t>
   </si>
   <si>
     <t>Mana Burst</t>
   </si>
   <si>
-    <t>Deal 3 damage</t>
-  </si>
-  <si>
     <t>Crystal Focus</t>
   </si>
   <si>
@@ -195,9 +141,6 @@
     <t>Spell Echo</t>
   </si>
   <si>
-    <t>Your next card triggers its base effect twice</t>
-  </si>
-  <si>
     <t>Mindstorm</t>
   </si>
   <si>
@@ -210,102 +153,48 @@
     <t>Golden Sprint</t>
   </si>
   <si>
-    <t>Heal 1</t>
-  </si>
-  <si>
     <t>Radiant Strike</t>
   </si>
   <si>
-    <t>Deal 2 damage and heal 1</t>
-  </si>
-  <si>
-    <t>Deal +2 damage</t>
-  </si>
-  <si>
     <t>Sunscale Guard</t>
   </si>
   <si>
-    <t>Gain 4 block</t>
-  </si>
-  <si>
-    <t>Gain 2 movement</t>
-  </si>
-  <si>
     <t>Swift Recovery</t>
   </si>
   <si>
-    <t>Heal 3</t>
-  </si>
-  <si>
     <t>Blinding Dash</t>
   </si>
   <si>
-    <t>Your next attack deals +2 damage</t>
-  </si>
-  <si>
     <t>Beacon Pulse</t>
   </si>
   <si>
-    <t>Heal 2 and draw 1 card</t>
-  </si>
-  <si>
     <t>Winged Rescue</t>
   </si>
   <si>
-    <t>Move to any open space</t>
-  </si>
-  <si>
     <t>Renewing Flame</t>
   </si>
   <si>
-    <t>Heal 4</t>
-  </si>
-  <si>
     <t>Solar Charge</t>
   </si>
   <si>
-    <t>Gain 3 movement and deal 3 damage</t>
-  </si>
-  <si>
     <t>Sacred Path</t>
   </si>
   <si>
-    <t>Gain 6 movement</t>
-  </si>
-  <si>
     <t>Guardian Light</t>
   </si>
   <si>
-    <t>Gain 6 block</t>
-  </si>
-  <si>
     <t>Life Pulse</t>
   </si>
   <si>
-    <t>Heal 5</t>
-  </si>
-  <si>
     <t>Sunflare Wings</t>
   </si>
   <si>
-    <t>Gain 4 movement and draw 1 card</t>
-  </si>
-  <si>
     <t>Dawnstrike</t>
   </si>
   <si>
-    <t>Heal damage dealt</t>
-  </si>
-  <si>
     <t>Celestial Flight</t>
   </si>
   <si>
-    <t>Gain 8 movement</t>
-  </si>
-  <si>
-    <t>Your next 2 cards gain their boost effects</t>
-  </si>
-  <si>
     <t>Strike</t>
   </si>
   <si>
@@ -318,102 +207,48 @@
     <t>Recover</t>
   </si>
   <si>
-    <t>Your next 2 boosts cost 0 magic</t>
-  </si>
-  <si>
     <t>Perfect Flow</t>
   </si>
   <si>
-    <t>Reveal top card: if pink, deal +5 damage</t>
-  </si>
-  <si>
     <t>Jackpot Breath</t>
   </si>
   <si>
-    <t>Lose 1 health to draw 2 cards</t>
-  </si>
-  <si>
     <t>Adrenaline Rush</t>
   </si>
   <si>
-    <t>Deal damage equal to cards played this turn</t>
-  </si>
-  <si>
     <t>Combo Finisher</t>
   </si>
   <si>
-    <t>If discarded card was pink, gain 1 magic</t>
-  </si>
-  <si>
-    <t>Draw 2 then discard 1</t>
-  </si>
-  <si>
     <t>Improvised Maneuver</t>
   </si>
   <si>
-    <t>If boosted, deal 2 damage again to another target</t>
-  </si>
-  <si>
     <t>Ricochet Claws</t>
   </si>
   <si>
-    <t>If another movement card was played this turn, gain 2 magic</t>
-  </si>
-  <si>
     <t>Slipstream</t>
   </si>
   <si>
-    <t>Gain 1 magic for each card played this turn</t>
-  </si>
-  <si>
     <t>Momentum Surge</t>
   </si>
   <si>
-    <t>50% chance to deal +4 damage</t>
-  </si>
-  <si>
     <t>Wild Swing</t>
   </si>
   <si>
-    <t>Your next card's base effect triggers twice</t>
-  </si>
-  <si>
     <t>Encore</t>
   </si>
   <si>
-    <t>Gain +2 movement</t>
-  </si>
-  <si>
-    <t>Gain 2 movement and 1 magic</t>
-  </si>
-  <si>
     <t>Flash Rhythm</t>
   </si>
   <si>
-    <t>If this is your third card this turn, attack a third time</t>
-  </si>
-  <si>
-    <t>Deal 1 damage twice</t>
-  </si>
-  <si>
     <t>Chain Assault</t>
   </si>
   <si>
-    <t>Reveal top card of deck. If pink, draw another card</t>
-  </si>
-  <si>
     <t>Lucky Break</t>
   </si>
   <si>
-    <t>If boosted, draw 1 card</t>
-  </si>
-  <si>
     <t>Flowstep</t>
   </si>
   <si>
-    <t>If another card was played this turn, deal +2 damage</t>
-  </si>
-  <si>
     <t>Momentum Strike</t>
   </si>
   <si>
@@ -516,10 +351,67 @@
     <t>Deal 3 {attack} to all {enemy}.</t>
   </si>
   <si>
-    <t>Search your discards for a card and draw it.</t>
-  </si>
-  <si>
-    <t>Your next Boost is free.</t>
+    <t>Plus 1 {attack} for each {pink} {card}.</t>
+  </si>
+  <si>
+    <t>Reveal the top {card}; If {pink}, draw it and another {card}.</t>
+  </si>
+  <si>
+    <t>Deal 1 {attack} to 2 {enemy}.</t>
+  </si>
+  <si>
+    <t>Reveal the top {card}; add it's power to the {attack}.</t>
+  </si>
+  <si>
+    <t>Flip a card; if it lands face up add 4 {attack}.</t>
+  </si>
+  <si>
+    <t>Lose 1 {health} to draw 2 {card}.</t>
+  </si>
+  <si>
+    <t>If another {movement} {card} was played this turn, gain 2 {magic}.</t>
+  </si>
+  <si>
+    <t>Deal 2 {attack} to a second {enemy} of your choice.</t>
+  </si>
+  <si>
+    <t>If discarded {card} was {pink}, gain 1 {magic}</t>
+  </si>
+  <si>
+    <t>Reveal top {card}; if {pink}, deal +5 {attack}.</t>
+  </si>
+  <si>
+    <t>Activate your next card twice.</t>
+  </si>
+  <si>
+    <t>Search your {discards} for a {card} and draw it.</t>
+  </si>
+  <si>
+    <t>Ignore {enemy} zones this turn</t>
+  </si>
+  <si>
+    <t>Your next {boost} is free.</t>
+  </si>
+  <si>
+    <t>{move} to any open space</t>
+  </si>
+  <si>
+    <t>Your next 2 {card} gain their {boost} effects.</t>
+  </si>
+  <si>
+    <t>Activate your next {card} twice.</t>
+  </si>
+  <si>
+    <t>Gain 1 {magic} for each {card} played this turn.</t>
+  </si>
+  <si>
+    <t>Draw 2 {card} then discard 1 {card}.</t>
+  </si>
+  <si>
+    <t>Deal {attack} equal to {card} played this turn.</t>
+  </si>
+  <si>
+    <t>Your next 2 {boost} are free.</t>
   </si>
 </sst>
 </file>
@@ -578,6 +470,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -893,43 +789,43 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>146</v>
+        <v>91</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>147</v>
+        <v>92</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>148</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -937,7 +833,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>89</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -967,7 +863,7 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -975,7 +871,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>143</v>
+        <v>88</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1005,7 +901,7 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1013,7 +909,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>87</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -1043,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1051,7 +947,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>86</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -1081,7 +977,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1089,7 +985,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>85</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -1119,7 +1015,7 @@
         <v>2</v>
       </c>
       <c r="M6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1127,7 +1023,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>139</v>
+        <v>84</v>
       </c>
       <c r="D7">
         <v>3</v>
@@ -1157,7 +1053,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -1165,7 +1061,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>83</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -1195,7 +1091,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1203,7 +1099,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -1233,7 +1129,7 @@
         <v>2</v>
       </c>
       <c r="M9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1241,7 +1137,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>81</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -1271,7 +1167,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1279,7 +1175,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>80</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -1309,7 +1205,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -1317,7 +1213,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>79</v>
       </c>
       <c r="D12">
         <v>4</v>
@@ -1347,7 +1243,7 @@
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1355,10 +1251,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>78</v>
       </c>
       <c r="C13" t="s">
-        <v>151</v>
+        <v>96</v>
       </c>
       <c r="D13">
         <v>5</v>
@@ -1388,7 +1284,7 @@
         <v>2</v>
       </c>
       <c r="M13" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1396,10 +1292,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>132</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>150</v>
+        <v>95</v>
       </c>
       <c r="D14">
         <v>4</v>
@@ -1429,7 +1325,7 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1437,7 +1333,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>131</v>
+        <v>76</v>
       </c>
       <c r="D15">
         <v>5</v>
@@ -1467,13 +1363,13 @@
         <v>3</v>
       </c>
       <c r="M15" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N15">
         <v>1</v>
       </c>
       <c r="O15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1481,7 +1377,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D16">
         <v>5</v>
@@ -1511,7 +1407,7 @@
         <v>3</v>
       </c>
       <c r="M16" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1549,43 +1445,43 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>146</v>
+        <v>91</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>147</v>
+        <v>92</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>148</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1593,10 +1489,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>152</v>
+        <v>97</v>
       </c>
       <c r="D2">
         <v>3</v>
@@ -1623,10 +1519,10 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M2" t="s">
-        <v>158</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1634,7 +1530,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>4</v>
@@ -1664,13 +1560,13 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N3">
         <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1678,7 +1574,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -1708,13 +1604,13 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N4">
         <v>2</v>
       </c>
       <c r="O4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1722,7 +1618,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D5">
         <v>5</v>
@@ -1749,10 +1645,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M5" t="s">
-        <v>155</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1760,7 +1656,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>3</v>
@@ -1790,7 +1686,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1798,10 +1694,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>98</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -1828,10 +1724,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M7" t="s">
-        <v>161</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -1839,7 +1735,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D8">
         <v>6</v>
@@ -1869,13 +1765,13 @@
         <v>2</v>
       </c>
       <c r="M8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N8">
         <v>3</v>
       </c>
       <c r="O8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1883,7 +1779,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D9">
         <v>3</v>
@@ -1910,10 +1806,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M9" t="s">
-        <v>160</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1921,10 +1817,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>99</v>
       </c>
       <c r="D10">
         <v>5</v>
@@ -1954,7 +1850,7 @@
         <v>2</v>
       </c>
       <c r="M10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1962,10 +1858,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="D11">
         <v>5</v>
@@ -1992,10 +1888,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M11" t="s">
-        <v>159</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2003,7 +1899,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D12">
         <v>5</v>
@@ -2033,13 +1929,13 @@
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N12">
         <v>2</v>
       </c>
       <c r="O12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -2047,7 +1943,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D13">
         <v>6</v>
@@ -2077,7 +1973,7 @@
         <v>5</v>
       </c>
       <c r="M13" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -2085,7 +1981,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D14">
         <v>5</v>
@@ -2115,7 +2011,7 @@
         <v>4</v>
       </c>
       <c r="M14" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -2123,10 +2019,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>156</v>
+        <v>101</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -2153,16 +2049,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M15" t="s">
-        <v>158</v>
+        <v>103</v>
       </c>
       <c r="N15">
         <v>2</v>
       </c>
       <c r="O15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -2170,10 +2066,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
-        <v>157</v>
+        <v>102</v>
       </c>
       <c r="D16">
         <v>8</v>
@@ -2200,10 +2096,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M16" t="s">
-        <v>162</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2235,37 +2131,37 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>146</v>
+        <v>91</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2273,7 +2169,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -2303,7 +2199,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2311,7 +2207,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -2341,7 +2237,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -2349,7 +2245,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -2379,7 +2275,7 @@
         <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2387,7 +2283,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -2417,7 +2313,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -2425,7 +2321,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>3</v>
@@ -2455,7 +2351,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2463,7 +2359,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -2490,10 +2386,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M7" t="s">
-        <v>48</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -2501,10 +2397,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>163</v>
+        <v>119</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -2534,7 +2430,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -2542,7 +2438,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -2572,7 +2468,7 @@
         <v>3</v>
       </c>
       <c r="M9" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -2580,7 +2476,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -2610,7 +2506,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -2618,7 +2514,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="D11">
         <v>4</v>
@@ -2648,7 +2544,7 @@
         <v>2</v>
       </c>
       <c r="M11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -2656,7 +2552,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="D12">
         <v>3</v>
@@ -2686,7 +2582,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -2694,10 +2590,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="D13">
         <v>6</v>
@@ -2727,7 +2623,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -2735,7 +2631,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="D14">
         <v>5</v>
@@ -2765,7 +2661,7 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -2773,7 +2669,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="D15">
         <v>6</v>
@@ -2803,7 +2699,7 @@
         <v>2</v>
       </c>
       <c r="M15" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -2811,7 +2707,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="D16">
         <v>7</v>
@@ -2838,10 +2734,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="M16" t="s">
-        <v>164</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2856,13 +2752,13 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="13" width="12" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="8" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="11" width="12" customWidth="1"/>
+    <col min="13" max="13" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -2873,7 +2769,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -2900,10 +2796,10 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2911,25 +2807,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="s">
-        <v>61</v>
+        <v>41</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -2938,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2952,40 +2845,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E3" t="s">
-        <v>64</v>
+        <v>42</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -2993,28 +2883,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" t="s">
-        <v>67</v>
+        <v>43</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -3023,10 +2910,10 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3034,40 +2921,37 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" t="s">
-        <v>67</v>
+        <v>44</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -3075,25 +2959,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" t="s">
-        <v>71</v>
+        <v>45</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -3105,10 +2986,10 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M6" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3116,40 +2997,37 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" t="s">
-        <v>41</v>
+        <v>46</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
-      <c r="M7">
-        <v>0</v>
+      <c r="M7" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -3157,25 +3035,25 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" t="s">
-        <v>28</v>
+        <v>122</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -3184,13 +3062,13 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -3198,19 +3076,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
+        <v>48</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -3219,19 +3094,19 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M9" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3239,25 +3114,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" t="s">
-        <v>28</v>
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -3266,13 +3138,13 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -3280,25 +3152,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E11" t="s">
-        <v>38</v>
+        <v>50</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -3312,8 +3181,8 @@
       <c r="L11">
         <v>2</v>
       </c>
-      <c r="M11">
-        <v>0</v>
+      <c r="M11" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -3321,40 +3190,37 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" t="s">
-        <v>83</v>
-      </c>
-      <c r="E12" t="s">
-        <v>69</v>
+        <v>51</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="M12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -3362,19 +3228,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" t="s">
-        <v>85</v>
-      </c>
-      <c r="E13" t="s">
-        <v>43</v>
+        <v>52</v>
+      </c>
+      <c r="D13">
+        <v>6</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -3383,19 +3246,19 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M13" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -3403,40 +3266,37 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E14" t="s">
-        <v>61</v>
+        <v>53</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -3444,22 +3304,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15">
         <v>6</v>
       </c>
-      <c r="D15" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" t="s">
-        <v>89</v>
+      <c r="E15">
+        <v>5</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -3471,13 +3328,13 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="M15" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -3485,16 +3342,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" t="s">
-        <v>91</v>
-      </c>
-      <c r="E16" t="s">
-        <v>92</v>
+        <v>55</v>
+      </c>
+      <c r="D16">
+        <v>8</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
       </c>
       <c r="F16">
         <v>8</v>
@@ -3503,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -3514,11 +3368,11 @@
       <c r="K16">
         <v>0</v>
       </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
+      <c r="L16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M16" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3533,14 +3387,13 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="44" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="13" width="12" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="8" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="11" width="12" customWidth="1"/>
+    <col min="13" max="13" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -3551,7 +3404,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -3578,10 +3431,10 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3589,22 +3442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E2" t="s">
-        <v>128</v>
+        <v>74</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -3618,11 +3468,11 @@
       <c r="K2">
         <v>0</v>
       </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
+      <c r="L2" t="s">
+        <v>94</v>
+      </c>
+      <c r="M2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3630,40 +3480,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
         <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" t="s">
-        <v>126</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -3671,40 +3518,37 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" t="s">
-        <v>124</v>
+        <v>72</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
+      <c r="L4" t="s">
+        <v>94</v>
+      </c>
+      <c r="M4" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3712,22 +3556,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E5" t="s">
-        <v>121</v>
+        <v>110</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -3741,11 +3585,11 @@
       <c r="K5">
         <v>0</v>
       </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
+      <c r="L5" t="s">
+        <v>94</v>
+      </c>
+      <c r="M5" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -3753,40 +3597,37 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E6" t="s">
-        <v>118</v>
+        <v>70</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3794,19 +3635,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
+        <v>124</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -3818,16 +3659,16 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -3835,22 +3676,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>114</v>
+        <v>68</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -3864,11 +3702,11 @@
       <c r="K8">
         <v>0</v>
       </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
+      <c r="L8" t="s">
+        <v>94</v>
+      </c>
+      <c r="M8" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -3876,19 +3714,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>113</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>112</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
+        <v>125</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -3900,16 +3738,16 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>3</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3917,16 +3755,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" t="s">
-        <v>110</v>
+        <v>66</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
       </c>
       <c r="F10">
         <v>5</v>
@@ -3935,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -3946,11 +3781,11 @@
       <c r="K10">
         <v>0</v>
       </c>
-      <c r="L10">
-        <v>2</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
+      <c r="L10" t="s">
+        <v>94</v>
+      </c>
+      <c r="M10" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -3958,22 +3793,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
-      </c>
-      <c r="C11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
-        <v>45</v>
-      </c>
-      <c r="E11" t="s">
-        <v>108</v>
+        <v>65</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -3987,11 +3819,11 @@
       <c r="K11">
         <v>0</v>
       </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
+      <c r="L11" t="s">
+        <v>94</v>
+      </c>
+      <c r="M11" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -3999,19 +3831,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" t="s">
-        <v>106</v>
-      </c>
-      <c r="E12" t="s">
-        <v>105</v>
+        <v>126</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -4023,16 +3855,16 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12">
         <v>0</v>
       </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
+      <c r="L12" t="s">
+        <v>94</v>
+      </c>
+      <c r="M12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -4040,19 +3872,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13">
         <v>6</v>
       </c>
-      <c r="D13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E13" t="s">
-        <v>14</v>
+      <c r="E13">
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -4070,10 +3902,10 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="M13" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -4081,19 +3913,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>102</v>
-      </c>
-      <c r="C14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" t="s">
-        <v>101</v>
+        <v>62</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -4110,11 +3939,11 @@
       <c r="K14">
         <v>0</v>
       </c>
-      <c r="L14">
-        <v>2</v>
-      </c>
-      <c r="M14">
-        <v>1</v>
+      <c r="L14" t="s">
+        <v>94</v>
+      </c>
+      <c r="M14" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -4122,22 +3951,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D15">
         <v>6</v>
       </c>
-      <c r="D15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" t="s">
-        <v>99</v>
+      <c r="E15">
+        <v>3</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -4151,11 +3977,11 @@
       <c r="K15">
         <v>0</v>
       </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
+      <c r="L15" t="s">
+        <v>94</v>
+      </c>
+      <c r="M15" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -4163,19 +3989,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" t="s">
-        <v>97</v>
-      </c>
-      <c r="E16" t="s">
-        <v>43</v>
+        <v>128</v>
+      </c>
+      <c r="D16">
+        <v>8</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -4187,16 +4013,16 @@
         <v>0</v>
       </c>
       <c r="J16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
       <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="M16" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4206,21 +4032,19 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="13" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="8" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4228,57 +4052,51 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>45</v>
+        <v>56</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -4289,37 +4107,31 @@
       <c r="J2">
         <v>0</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>40</v>
+        <v>57</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -4327,34 +4139,28 @@
       <c r="J3">
         <v>0</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>22</v>
+        <v>58</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -4363,39 +4169,33 @@
         <v>0</v>
       </c>
       <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
+        <v>59</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -4403,48 +4203,36 @@
       <c r="J5">
         <v>0</v>
       </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
+        <v>90</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
         <v>0</v>
       </c>
     </row>

</xml_diff>